<commit_message>
feat(productos): Kit de Tareas Cafetería v2.0 (500 tareas) y Pizzería v2.0 (373) — motor de familia 2.4 + contenido propio; idempotencia 0, cache 143/139, censo 0, gate offline 11/11 cada uno
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-tareas-cafeteria/02-partidas-cocina.xlsx
+++ b/astro-site/public/dl/kit-tareas-cafeteria/02-partidas-cocina.xlsx
@@ -13,12 +13,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pastelería Vitrina" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Instrucciones'!$A$1:$B$33</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Calientes'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Calientes'!$A$1:$G$29</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Calientes'!$A$1:$G$36</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Fríos'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Fríos'!$A$1:$G$28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Fríos'!$A$1:$G$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Pastelería Vitrina'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Pastelería Vitrina'!$A$1:$G$33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Pastelería Vitrina'!$A$1:$G$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -27,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -91,8 +92,22 @@
       <color rgb="00666666"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFD700"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00333333"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="00555555"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -123,6 +138,11 @@
         <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -150,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -192,6 +212,50 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -569,72 +633,165 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1"/>
-    <row r="2">
-      <c r="B2" s="1" t="inlineStr">
+    <row r="2" ht="26" customHeight="1">
+      <c r="B2" s="22" t="inlineStr">
         <is>
           <t>Tareas por Partida de Cocina — Cafetería / Brunch</t>
         </is>
       </c>
     </row>
     <row r="3"/>
-    <row r="4">
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Checklists específicos para cada partida de cocina de cafetería/brunch.</t>
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="23" t="inlineStr">
+        <is>
+          <t>Cómo cuenta el contador</t>
         </is>
       </c>
     </row>
     <row r="5"/>
-    <row r="6">
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>• Cada pestaña cubre una partida diferente</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>• Las tareas están organizadas: antes, durante y después del servicio</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>• Imprime una por partida y entrégala al responsable</t>
+    <row r="6" ht="32" customHeight="1">
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>▸ Marca con ✓ en la columna «✓ Completada» (desplegable): es la que cuenta el total de tareas completadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>▸ «N/A» = no aplica en tu local: esa tarea SALE del total (no la borres, márcala N/A). «—» = no hecha: sigue contando como pendiente y baja el porcentaje, que es de lo que se trata.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>▸ El denominador cuenta las tareas escritas en la columna «Tarea», no un número fijo: si añades o borras tareas, el total se ajusta solo.</t>
         </is>
       </c>
     </row>
     <row r="9"/>
-    <row r="10">
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Formato: ☐ = tarea pendiente · ✓ = completada (escribe en columna 'Hecha')</t>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>Filas libres</t>
         </is>
       </c>
     </row>
     <row r="11"/>
-    <row r="12">
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Marca con ✓ en la columna «✓ Completada» (desplegable): es la que cuenta el total de tareas completadas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13"/>
+    <row r="12" ht="32" customHeight="1">
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>▸ Al final de cada tabla hay 5 filas verdes libres DENTRO del rango que cuenta el contador: escribe ahí tus tareas propias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>▸ Si necesitas más, inserta filas DENTRO de la tabla (clic derecho → Insertar), nunca por debajo de la última: lo que se escriba fuera del rango no lo cuenta nadie.</t>
+        </is>
+      </c>
+    </row>
     <row r="14">
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Versión 1.1 · agosto 2026 · aichef.pro/kit-tareas-cafeteria · info@aichef.pro</t>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>Protección de la hoja</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>▸ Las hojas con fórmulas van protegidas SIN contraseña: las celdas de entrada (las verdes) están desbloqueadas y los cálculos no se pisan por accidente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="B18" s="24" t="inlineStr">
+        <is>
+          <t>▸ Puedes insertar y borrar filas con la protección puesta. Para cambiar la estructura: Revisar → Desproteger hoja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="B20" s="23" t="inlineStr">
+        <is>
+          <t>Se conecta con</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="B22" s="24" t="inlineStr">
+        <is>
+          <t>▸ 08-apertura-cierre-negocio.xlsx — checklist del LOCAL completo: es el MARCO del día.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>▸ 01-apertura-cierre.xlsx — el mismo día con el DETALLE por área (cocina, sala, barra café).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="B24" s="24" t="inlineStr">
+        <is>
+          <t>▸ 09-apertura-cierre-caja.xlsx — la CAJA: fondo, recuento por denominaciones, Z del TPV y descuadre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="48" customHeight="1">
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t>▸ Orden de uso: local → áreas → caja. Cada fichero cubre un nivel: el de negocio marca el HITO (encender, abrir, cerrar), el de áreas detalla CÓMO se hace en cada zona y el de caja lleva el DINERO. Si una tarea aparece en dos, es a propósito: una es el hito y la otra el detalle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="B26" s="24" t="inlineStr">
+        <is>
+          <t>▸ Estás en 02-partidas-cocina.xlsx: es una capa MÁS, no una repetición — el marco del día está en 08-apertura-cierre-negocio.xlsx y 01-apertura-cierre.xlsx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="B28" s="23" t="inlineStr">
+        <is>
+          <t>— Kit de Tareas Recurrentes · Cafetería / Brunch · AI Chef Pro · aichef.pro</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="35" customHeight="1">
+      <c r="B30" s="23" t="inlineStr">
+        <is>
+          <t>Diseñado por John Guerrero — chef y consultor gastronómico desde 2010, en cocina desde los 17 años · johnguerrero.es</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="B31" s="23" t="inlineStr">
+        <is>
+          <t>Contacto: info@aichef.pro</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="B33" s="23" t="inlineStr">
+        <is>
+          <t>Versión 2.0 · agosto 2026 · aichef.pro/kit-tareas-cafeteria · info@aichef.pro</t>
         </is>
       </c>
     </row>
@@ -659,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -709,7 +866,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Hora Límite</t>
+          <t>Cuándo</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -724,512 +881,631 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  ANTES DEL SERVICIO</t>
         </is>
       </c>
+      <c r="B5" s="26" t="n"/>
+      <c r="C5" s="26" t="n"/>
+      <c r="D5" s="26" t="n"/>
+      <c r="E5" s="26" t="n"/>
+      <c r="F5" s="26" t="n"/>
+      <c r="G5" s="26" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="n">
+      <c r="A6" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="28" t="inlineStr">
         <is>
           <t>Encender y precalentar plancha para tostadas</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="C6" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D6" s="29" t="inlineStr">
         <is>
           <t>Cocinero calientes</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="E6" s="29" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="F6" s="11" t="n"/>
-      <c r="G6" s="11" t="n"/>
+      <c r="F6" s="30" t="n"/>
+      <c r="G6" s="30" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="n">
+      <c r="A7" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="32" t="inlineStr">
         <is>
           <t>Encender horno: precalentar para croissants y quiches</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="C7" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D7" s="29" t="inlineStr">
         <is>
           <t>Cocinero calientes</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E7" s="29" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="F7" s="15" t="n"/>
-      <c r="G7" s="15" t="n"/>
+      <c r="F7" s="30" t="n"/>
+      <c r="G7" s="30" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="n">
+      <c r="A8" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="28" t="inlineStr">
         <is>
           <t>Preparar mise en place: bacon, huevos, salmón ahumado</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="C8" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D8" s="29" t="inlineStr">
         <is>
           <t>Cocinero calientes</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="E8" s="29" t="inlineStr">
         <is>
           <t>07:15</t>
         </is>
       </c>
-      <c r="F8" s="11" t="n"/>
-      <c r="G8" s="11" t="n"/>
+      <c r="F8" s="30" t="n"/>
+      <c r="G8" s="30" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="n">
+      <c r="A9" s="27" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="28" t="inlineStr">
+        <is>
+          <t>Salmón ahumado y pescado que se sirve sin cocinar — prevención de ANISAKIS: exigir al proveedor el certificado de congelación previa (≥24 h a −20 °C o −35 °C 15 h) o congelarlo tú, y anotar el lote</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D9" s="29" t="inlineStr">
+        <is>
+          <t>Cocinero calientes</t>
+        </is>
+      </c>
+      <c r="E9" s="29" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="F9" s="30" t="n"/>
+      <c r="G9" s="30" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="31" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="32" t="inlineStr">
         <is>
           <t>Preparar batch de huevos revueltos base</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="C10" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D10" s="29" t="inlineStr">
         <is>
           <t>Cocinero calientes</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E10" s="29" t="inlineStr">
         <is>
           <t>07:15</t>
         </is>
       </c>
-      <c r="F9" s="15" t="n"/>
-      <c r="G9" s="15" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="F10" s="30" t="n"/>
+      <c r="G10" s="30" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="28" t="inlineStr">
         <is>
           <t>Preparar pancakes/tortitas: masa lista en jarra</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="C11" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D11" s="29" t="inlineStr">
         <is>
           <t>Cocinero calientes</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E11" s="29" t="inlineStr">
         <is>
           <t>07:15</t>
         </is>
       </c>
-      <c r="F10" s="11" t="n"/>
-      <c r="G10" s="11" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="21" t="n">
-        <v>6</v>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="F11" s="30" t="n"/>
+      <c r="G11" s="30" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="31" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="32" t="inlineStr">
         <is>
           <t>Cortar y tostar pan: sourdough, brioche, centeno</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D11" s="14" t="inlineStr">
+      <c r="C12" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="inlineStr">
         <is>
           <t>Cocinero calientes</t>
         </is>
       </c>
-      <c r="E11" s="14" t="inlineStr">
+      <c r="E12" s="29" t="inlineStr">
         <is>
           <t>07:30</t>
         </is>
       </c>
-      <c r="F11" s="15" t="n"/>
-      <c r="G11" s="15" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="20" t="n">
-        <v>7</v>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="F12" s="30" t="n"/>
+      <c r="G12" s="30" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="28" t="inlineStr">
         <is>
           <t>Verificar stock de mantequilla y aceite de oliva</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="C13" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D13" s="29" t="inlineStr">
         <is>
           <t>Cocinero calientes</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="E13" s="29" t="inlineStr">
         <is>
           <t>07:15</t>
         </is>
       </c>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="F13" s="30" t="n"/>
+      <c r="G13" s="30" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  DURANTE EL SERVICIO</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="20" t="n">
-        <v>8</v>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="26" t="n"/>
+      <c r="C14" s="26" t="n"/>
+      <c r="D14" s="26" t="n"/>
+      <c r="E14" s="26" t="n"/>
+      <c r="F14" s="26" t="n"/>
+      <c r="G14" s="26" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="27" t="n">
+        <v>9</v>
+      </c>
+      <c r="B15" s="28" t="inlineStr">
         <is>
           <t>Mantener plancha limpia entre comandas</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D15" s="29" t="inlineStr">
         <is>
           <t>Cocinero calientes</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="E15" s="29" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F14" s="11" t="n"/>
-      <c r="G14" s="11" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="21" t="n">
-        <v>9</v>
-      </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="F15" s="30" t="n"/>
+      <c r="G15" s="30" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="31" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" s="32" t="inlineStr">
         <is>
           <t>Controlar punto de huevos: pochados, revueltos, fritos</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D16" s="29" t="inlineStr">
         <is>
           <t>Cocinero calientes</t>
         </is>
       </c>
-      <c r="E15" s="14" t="inlineStr">
+      <c r="E16" s="29" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F15" s="15" t="n"/>
-      <c r="G15" s="15" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="20" t="n">
-        <v>10</v>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="F16" s="30" t="n"/>
+      <c r="G16" s="30" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="27" t="n">
+        <v>11</v>
+      </c>
+      <c r="B17" s="28" t="inlineStr">
         <is>
           <t>Reponer pan tostado según demanda</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="C17" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D17" s="29" t="inlineStr">
         <is>
           <t>Cocinero calientes</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="E17" s="29" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F16" s="11" t="n"/>
-      <c r="G16" s="11" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="21" t="n">
-        <v>11</v>
-      </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="F17" s="30" t="n"/>
+      <c r="G17" s="30" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="31" t="n">
+        <v>12</v>
+      </c>
+      <c r="B18" s="32" t="inlineStr">
         <is>
           <t>Hornear croissants/bollería por tandas</t>
         </is>
       </c>
-      <c r="C17" s="14" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="C18" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D18" s="29" t="inlineStr">
         <is>
           <t>Cocinero calientes</t>
         </is>
       </c>
-      <c r="E17" s="14" t="inlineStr">
+      <c r="E18" s="29" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F17" s="15" t="n"/>
-      <c r="G17" s="15" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="20" t="n">
-        <v>12</v>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="F18" s="30" t="n"/>
+      <c r="G18" s="30" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="27" t="n">
+        <v>13</v>
+      </c>
+      <c r="B19" s="28" t="inlineStr">
         <is>
           <t>Controlar tiempos de espera en pase</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D18" s="10" t="inlineStr">
+      <c r="C19" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D19" s="29" t="inlineStr">
         <is>
           <t>Cocinero calientes</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="E19" s="29" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F18" s="11" t="n"/>
-      <c r="G18" s="11" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="F19" s="30" t="n"/>
+      <c r="G19" s="30" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  DESPUÉS DEL SERVICIO</t>
         </is>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="20" t="n">
-        <v>13</v>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="26" t="n"/>
+      <c r="C20" s="26" t="n"/>
+      <c r="D20" s="26" t="n"/>
+      <c r="E20" s="26" t="n"/>
+      <c r="F20" s="26" t="n"/>
+      <c r="G20" s="26" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="27" t="n">
+        <v>14</v>
+      </c>
+      <c r="B21" s="28" t="inlineStr">
         <is>
           <t>Limpiar y desinfectar plancha</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
+      <c r="C21" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D21" s="29" t="inlineStr">
         <is>
           <t>Cocinero calientes</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="E21" s="29" t="inlineStr">
         <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="F20" s="11" t="n"/>
-      <c r="G20" s="11" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="21" t="n">
-        <v>14</v>
-      </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="F21" s="30" t="n"/>
+      <c r="G21" s="30" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="31" t="n">
+        <v>15</v>
+      </c>
+      <c r="B22" s="32" t="inlineStr">
         <is>
           <t>Guardar mise en place sobrante (etiquetar)</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="C22" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D22" s="29" t="inlineStr">
         <is>
           <t>Cocinero calientes</t>
         </is>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E22" s="29" t="inlineStr">
         <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="F21" s="15" t="n"/>
-      <c r="G21" s="15" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="20" t="n">
-        <v>15</v>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="F22" s="30" t="n"/>
+      <c r="G22" s="30" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="27" t="n">
+        <v>16</v>
+      </c>
+      <c r="B23" s="28" t="inlineStr">
         <is>
           <t>Limpiar horno si se usó</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D22" s="10" t="inlineStr">
+      <c r="C23" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D23" s="29" t="inlineStr">
         <is>
           <t>Cocinero calientes</t>
         </is>
       </c>
-      <c r="E22" s="10" t="inlineStr">
+      <c r="E23" s="29" t="inlineStr">
         <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="F22" s="11" t="n"/>
-      <c r="G22" s="11" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="21" t="n">
-        <v>16</v>
-      </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="F23" s="30" t="n"/>
+      <c r="G23" s="30" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="31" t="n">
+        <v>17</v>
+      </c>
+      <c r="B24" s="32" t="inlineStr">
         <is>
           <t>Anotar consumos del día para pedidos</t>
         </is>
       </c>
-      <c r="C23" s="14" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="C24" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D24" s="29" t="inlineStr">
         <is>
           <t>Cocinero calientes</t>
         </is>
       </c>
-      <c r="E23" s="14" t="inlineStr">
+      <c r="E24" s="29" t="inlineStr">
         <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="F23" s="15" t="n"/>
-      <c r="G23" s="15" t="n"/>
-    </row>
-    <row r="24"/>
+      <c r="F24" s="30" t="n"/>
+      <c r="G24" s="30" t="n"/>
+    </row>
     <row r="25">
-      <c r="C25" s="16" t="inlineStr">
-        <is>
-          <t>Completadas:</t>
-        </is>
-      </c>
-      <c r="D25" s="17">
-        <f>COUNTIF(F5:F23,"✓")</f>
+      <c r="A25" s="31" t="n">
+        <v>18</v>
+      </c>
+      <c r="B25" s="32" t="inlineStr">
+        <is>
+          <t>Anotar las mermas del turno (producto, cantidad y motivo): sin este dato el food cost del mes sale mal</t>
+        </is>
+      </c>
+      <c r="C25" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D25" s="29" t="inlineStr">
+        <is>
+          <t>Cocinero calientes</t>
+        </is>
+      </c>
+      <c r="E25" s="29" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="F25" s="30" t="n"/>
+      <c r="G25" s="30" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="33" t="n"/>
+      <c r="B26" s="34" t="n"/>
+      <c r="C26" s="29" t="n"/>
+      <c r="D26" s="29" t="n"/>
+      <c r="E26" s="29" t="n"/>
+      <c r="F26" s="30" t="n"/>
+      <c r="G26" s="30" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="33" t="n"/>
+      <c r="B27" s="34" t="n"/>
+      <c r="C27" s="29" t="n"/>
+      <c r="D27" s="29" t="n"/>
+      <c r="E27" s="29" t="n"/>
+      <c r="F27" s="30" t="n"/>
+      <c r="G27" s="30" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="33" t="n"/>
+      <c r="B28" s="34" t="n"/>
+      <c r="C28" s="29" t="n"/>
+      <c r="D28" s="29" t="n"/>
+      <c r="E28" s="29" t="n"/>
+      <c r="F28" s="30" t="n"/>
+      <c r="G28" s="30" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="33" t="n"/>
+      <c r="B29" s="34" t="n"/>
+      <c r="C29" s="29" t="n"/>
+      <c r="D29" s="29" t="n"/>
+      <c r="E29" s="29" t="n"/>
+      <c r="F29" s="30" t="n"/>
+      <c r="G29" s="30" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="33" t="n"/>
+      <c r="B30" s="34" t="n"/>
+      <c r="C30" s="29" t="n"/>
+      <c r="D30" s="29" t="n"/>
+      <c r="E30" s="29" t="n"/>
+      <c r="F30" s="30" t="n"/>
+      <c r="G30" s="30" t="n"/>
+    </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>Tareas completadas:</t>
+        </is>
+      </c>
+      <c r="D32" s="17">
+        <f>COUNTIFS(B5:B30,"?*",F5:F30,"✓")</f>
         <v>0.0</v>
       </c>
-      <c r="E25" s="16" t="inlineStr">
+      <c r="E32" s="16" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="F25">
-        <f>COUNTIF(B5:B23,"?*")</f>
-        <v>16.0</v>
-      </c>
-    </row>
-    <row r="26"/>
-    <row r="27">
-      <c r="A27" s="18" t="inlineStr">
+      <c r="F32">
+        <f>COUNTIF(B5:B30,"?*")-COUNTIF(F5:F30,"N/A")</f>
+        <v>18.0</v>
+      </c>
+    </row>
+    <row r="33"/>
+    <row r="34">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t>Firma encargado/a: _________________________    Hora: _________</t>
         </is>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29">
-      <c r="A29" s="19" t="inlineStr">
-        <is>
-          <t>— Kit de Tareas Recurrentes: Cafetería / Brunch · AI Chef Pro · aichef.pro —</t>
+    <row r="35"/>
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>— Kit de Tareas Recurrentes · Cafetería / Brunch · AI Chef Pro · aichef.pro</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="0"/>
+  <mergeCells count="8">
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A36:G36"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A27:G27"/>
-    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A32:C32"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="A14:G14"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A19:G19"/>
-    <mergeCell ref="A29:G29"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:G23">
+  <conditionalFormatting sqref="A5:G30">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$F5="✓"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F12 F14 F15 F16 F17 F18 F20 F21 F22 F23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F12 F13 F15 F16 F17 F18 F19 F21 F22 F23 F24 F25 F26 F27 F28 F29 F30" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." type="list" errorStyle="stop">
       <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1253,7 +1529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1303,7 +1579,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Hora Límite</t>
+          <t>Cuándo</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -1318,485 +1594,577 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  ANTES DEL SERVICIO</t>
         </is>
       </c>
+      <c r="B5" s="26" t="n"/>
+      <c r="C5" s="26" t="n"/>
+      <c r="D5" s="26" t="n"/>
+      <c r="E5" s="26" t="n"/>
+      <c r="F5" s="26" t="n"/>
+      <c r="G5" s="26" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="n">
+      <c r="A6" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Lavar y desinfectar vegetales frescos</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="B6" s="28" t="inlineStr">
+        <is>
+          <t>Lavar y desinfectar las hojas verdes y los vegetales que se sirven crudos con lejía apta para uso alimentario según la dosis del fabricante (habitual: 70 ppm, 5 min) y ACLARAR con agua potable abundante</t>
+        </is>
+      </c>
+      <c r="C6" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D6" s="29" t="inlineStr">
         <is>
           <t>Cocinero fríos</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="E6" s="29" t="inlineStr">
         <is>
           <t>07:15</t>
         </is>
       </c>
-      <c r="F6" s="11" t="n"/>
-      <c r="G6" s="11" t="n"/>
+      <c r="F6" s="30" t="n"/>
+      <c r="G6" s="30" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="n">
+      <c r="A7" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="32" t="inlineStr">
         <is>
           <t>Preparar base de açaí bowls</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="C7" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D7" s="29" t="inlineStr">
         <is>
           <t>Cocinero fríos</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E7" s="29" t="inlineStr">
         <is>
           <t>07:15</t>
         </is>
       </c>
-      <c r="F7" s="15" t="n"/>
-      <c r="G7" s="15" t="n"/>
+      <c r="F7" s="30" t="n"/>
+      <c r="G7" s="30" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="n">
+      <c r="A8" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="28" t="inlineStr">
         <is>
           <t>Cortar fruta fresca: plátano, fresa, mango, arándanos</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="C8" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D8" s="29" t="inlineStr">
         <is>
           <t>Cocinero fríos</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="E8" s="29" t="inlineStr">
         <is>
           <t>07:15</t>
         </is>
       </c>
-      <c r="F8" s="11" t="n"/>
-      <c r="G8" s="11" t="n"/>
+      <c r="F8" s="30" t="n"/>
+      <c r="G8" s="30" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="n">
+      <c r="A9" s="31" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="32" t="inlineStr">
         <is>
           <t>Preparar granola casera o verificar stock</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="C9" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D9" s="29" t="inlineStr">
         <is>
           <t>Cocinero fríos</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="29" t="inlineStr">
         <is>
           <t>07:15</t>
         </is>
       </c>
-      <c r="F9" s="15" t="n"/>
-      <c r="G9" s="15" t="n"/>
+      <c r="F9" s="30" t="n"/>
+      <c r="G9" s="30" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="n">
+      <c r="A10" s="27" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="28" t="inlineStr">
         <is>
           <t>Preparar overnight oats (si se hacen en el momento)</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="C10" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D10" s="29" t="inlineStr">
         <is>
           <t>Cocinero fríos</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E10" s="29" t="inlineStr">
         <is>
           <t>07:15</t>
         </is>
       </c>
-      <c r="F10" s="11" t="n"/>
-      <c r="G10" s="11" t="n"/>
+      <c r="F10" s="30" t="n"/>
+      <c r="G10" s="30" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="n">
+      <c r="A11" s="31" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="32" t="inlineStr">
         <is>
           <t>Machacar aguacate fresco para smashed avocado</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D11" s="14" t="inlineStr">
+      <c r="C11" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D11" s="29" t="inlineStr">
         <is>
           <t>Cocinero fríos</t>
         </is>
       </c>
-      <c r="E11" s="14" t="inlineStr">
+      <c r="E11" s="29" t="inlineStr">
         <is>
           <t>07:30</t>
         </is>
       </c>
-      <c r="F11" s="15" t="n"/>
-      <c r="G11" s="15" t="n"/>
+      <c r="F11" s="30" t="n"/>
+      <c r="G11" s="30" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="n">
+      <c r="A12" s="27" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="28" t="inlineStr">
         <is>
           <t>Preparar ensaladas base para menú del día</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="C12" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="inlineStr">
         <is>
           <t>Cocinero fríos</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="E12" s="29" t="inlineStr">
         <is>
           <t>07:30</t>
         </is>
       </c>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n"/>
+      <c r="F12" s="30" t="n"/>
+      <c r="G12" s="30" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  DURANTE EL SERVICIO</t>
         </is>
       </c>
+      <c r="B13" s="26" t="n"/>
+      <c r="C13" s="26" t="n"/>
+      <c r="D13" s="26" t="n"/>
+      <c r="E13" s="26" t="n"/>
+      <c r="F13" s="26" t="n"/>
+      <c r="G13" s="26" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="20" t="n">
+      <c r="A14" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="28" t="inlineStr">
         <is>
           <t>Montar bowls al momento: base + toppings + salsa</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="C14" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D14" s="29" t="inlineStr">
         <is>
           <t>Cocinero fríos</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="E14" s="29" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F14" s="11" t="n"/>
-      <c r="G14" s="11" t="n"/>
+      <c r="F14" s="30" t="n"/>
+      <c r="G14" s="30" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="n">
+      <c r="A15" s="31" t="n">
         <v>9</v>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="32" t="inlineStr">
         <is>
           <t>Mantener toppings frescos (cubrir cuando no se usan)</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D15" s="29" t="inlineStr">
         <is>
           <t>Cocinero fríos</t>
         </is>
       </c>
-      <c r="E15" s="14" t="inlineStr">
+      <c r="E15" s="29" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F15" s="15" t="n"/>
-      <c r="G15" s="15" t="n"/>
+      <c r="F15" s="30" t="n"/>
+      <c r="G15" s="30" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="n">
+      <c r="A16" s="27" t="n">
         <v>10</v>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="28" t="inlineStr">
         <is>
           <t>Reponer inserts de fruta y vegetales según se agoten</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D16" s="29" t="inlineStr">
         <is>
           <t>Cocinero fríos</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="E16" s="29" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F16" s="11" t="n"/>
-      <c r="G16" s="11" t="n"/>
+      <c r="F16" s="30" t="n"/>
+      <c r="G16" s="30" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="n">
+      <c r="A17" s="31" t="n">
         <v>11</v>
       </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>Controlar temperatura de cámara de ingredientes fríos</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="B17" s="32" t="inlineStr">
+        <is>
+          <t>Controlar temperatura de cámara de ingredientes fríos (refrigeración 0-4 °C) — anota la lectura: ____ °C</t>
+        </is>
+      </c>
+      <c r="C17" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D17" s="29" t="inlineStr">
         <is>
           <t>Cocinero fríos</t>
         </is>
       </c>
-      <c r="E17" s="14" t="inlineStr">
+      <c r="E17" s="29" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F17" s="15" t="n"/>
-      <c r="G17" s="15" t="n"/>
+      <c r="F17" s="30" t="n"/>
+      <c r="G17" s="30" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  DESPUÉS DEL SERVICIO</t>
         </is>
       </c>
+      <c r="B18" s="26" t="n"/>
+      <c r="C18" s="26" t="n"/>
+      <c r="D18" s="26" t="n"/>
+      <c r="E18" s="26" t="n"/>
+      <c r="F18" s="26" t="n"/>
+      <c r="G18" s="26" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="21" t="n">
+      <c r="A19" s="31" t="n">
         <v>12</v>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B19" s="32" t="inlineStr">
         <is>
           <t>Cubrir y refrigerar todos los inserts</t>
         </is>
       </c>
-      <c r="C19" s="14" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D19" s="14" t="inlineStr">
+      <c r="C19" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D19" s="29" t="inlineStr">
         <is>
           <t>Cocinero fríos</t>
         </is>
       </c>
-      <c r="E19" s="14" t="inlineStr">
+      <c r="E19" s="29" t="inlineStr">
         <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="F19" s="15" t="n"/>
-      <c r="G19" s="15" t="n"/>
+      <c r="F19" s="30" t="n"/>
+      <c r="G19" s="30" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="20" t="n">
+      <c r="A20" s="27" t="n">
         <v>13</v>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="28" t="inlineStr">
         <is>
           <t>Desechar fruta cortada que lleve +24h</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
+      <c r="C20" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D20" s="29" t="inlineStr">
         <is>
           <t>Cocinero fríos</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="E20" s="29" t="inlineStr">
         <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="F20" s="11" t="n"/>
-      <c r="G20" s="11" t="n"/>
+      <c r="F20" s="30" t="n"/>
+      <c r="G20" s="30" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="21" t="n">
+      <c r="A21" s="31" t="n">
         <v>14</v>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="32" t="inlineStr">
         <is>
           <t>Limpiar y desinfectar tablas y cuchillos</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="C21" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D21" s="29" t="inlineStr">
         <is>
           <t>Cocinero fríos</t>
         </is>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E21" s="29" t="inlineStr">
         <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="F21" s="15" t="n"/>
-      <c r="G21" s="15" t="n"/>
+      <c r="F21" s="30" t="n"/>
+      <c r="G21" s="30" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="20" t="n">
+      <c r="A22" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="28" t="inlineStr">
         <is>
           <t>Anotar consumos para pedidos</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D22" s="10" t="inlineStr">
+      <c r="C22" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D22" s="29" t="inlineStr">
         <is>
           <t>Cocinero fríos</t>
         </is>
       </c>
-      <c r="E22" s="10" t="inlineStr">
+      <c r="E22" s="29" t="inlineStr">
         <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="F22" s="11" t="n"/>
-      <c r="G22" s="11" t="n"/>
-    </row>
-    <row r="23"/>
+      <c r="F22" s="30" t="n"/>
+      <c r="G22" s="30" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="27" t="n">
+        <v>16</v>
+      </c>
+      <c r="B23" s="28" t="inlineStr">
+        <is>
+          <t>Anotar las mermas del turno: fruta cortada, aguacate y bowls montados que no se han vendido</t>
+        </is>
+      </c>
+      <c r="C23" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D23" s="29" t="inlineStr">
+        <is>
+          <t>Cocinero fríos</t>
+        </is>
+      </c>
+      <c r="E23" s="29" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="F23" s="30" t="n"/>
+      <c r="G23" s="30" t="n"/>
+    </row>
     <row r="24">
-      <c r="C24" s="16" t="inlineStr">
-        <is>
-          <t>Completadas:</t>
-        </is>
-      </c>
-      <c r="D24" s="17">
-        <f>COUNTIF(F5:F22,"✓")</f>
+      <c r="A24" s="33" t="n"/>
+      <c r="B24" s="34" t="n"/>
+      <c r="C24" s="29" t="n"/>
+      <c r="D24" s="29" t="n"/>
+      <c r="E24" s="29" t="n"/>
+      <c r="F24" s="30" t="n"/>
+      <c r="G24" s="30" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="33" t="n"/>
+      <c r="B25" s="34" t="n"/>
+      <c r="C25" s="29" t="n"/>
+      <c r="D25" s="29" t="n"/>
+      <c r="E25" s="29" t="n"/>
+      <c r="F25" s="30" t="n"/>
+      <c r="G25" s="30" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="33" t="n"/>
+      <c r="B26" s="34" t="n"/>
+      <c r="C26" s="29" t="n"/>
+      <c r="D26" s="29" t="n"/>
+      <c r="E26" s="29" t="n"/>
+      <c r="F26" s="30" t="n"/>
+      <c r="G26" s="30" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="33" t="n"/>
+      <c r="B27" s="34" t="n"/>
+      <c r="C27" s="29" t="n"/>
+      <c r="D27" s="29" t="n"/>
+      <c r="E27" s="29" t="n"/>
+      <c r="F27" s="30" t="n"/>
+      <c r="G27" s="30" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="33" t="n"/>
+      <c r="B28" s="34" t="n"/>
+      <c r="C28" s="29" t="n"/>
+      <c r="D28" s="29" t="n"/>
+      <c r="E28" s="29" t="n"/>
+      <c r="F28" s="30" t="n"/>
+      <c r="G28" s="30" t="n"/>
+    </row>
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t>Tareas completadas:</t>
+        </is>
+      </c>
+      <c r="D30" s="17">
+        <f>COUNTIFS(B5:B28,"?*",F5:F28,"✓")</f>
         <v>0.0</v>
       </c>
-      <c r="E24" s="16" t="inlineStr">
+      <c r="E30" s="16" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="F24">
-        <f>COUNTIF(B5:B22,"?*")</f>
-        <v>15.0</v>
-      </c>
-    </row>
-    <row r="25"/>
-    <row r="26">
-      <c r="A26" s="18" t="inlineStr">
+      <c r="F30">
+        <f>COUNTIF(B5:B28,"?*")-COUNTIF(F5:F28,"N/A")</f>
+        <v>16.0</v>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr">
         <is>
           <t>Firma encargado/a: _________________________    Hora: _________</t>
         </is>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28">
-      <c r="A28" s="19" t="inlineStr">
-        <is>
-          <t>— Kit de Tareas Recurrentes: Cafetería / Brunch · AI Chef Pro · aichef.pro —</t>
+    <row r="33"/>
+    <row r="34">
+      <c r="A34" s="19" t="inlineStr">
+        <is>
+          <t>— Kit de Tareas Recurrentes · Cafetería / Brunch · AI Chef Pro · aichef.pro</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A28:G28"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="0"/>
+  <mergeCells count="8">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A34:G34"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A30:C30"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A26:G26"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:G22">
+  <conditionalFormatting sqref="A5:G28">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$F5="✓"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F12 F14 F15 F16 F17 F19 F20 F21 F22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F12 F14 F15 F16 F17 F19 F20 F21 F22 F23 F24 F25 F26 F27 F28" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." type="list" errorStyle="stop">
       <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1820,7 +2188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1870,7 +2238,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Hora Límite</t>
+          <t>Cuándo</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -1885,601 +2253,672 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  PRODUCCIÓN MATUTINA</t>
         </is>
       </c>
+      <c r="B5" s="26" t="n"/>
+      <c r="C5" s="26" t="n"/>
+      <c r="D5" s="26" t="n"/>
+      <c r="E5" s="26" t="n"/>
+      <c r="F5" s="26" t="n"/>
+      <c r="G5" s="26" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="n">
+      <c r="A6" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="28" t="inlineStr">
         <is>
           <t>Hornear croissants, magdalenas, muffins del día</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="C6" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D6" s="29" t="inlineStr">
         <is>
           <t>Pastelero/a</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="E6" s="29" t="inlineStr">
         <is>
           <t>06:30</t>
         </is>
       </c>
-      <c r="F6" s="11" t="n"/>
-      <c r="G6" s="11" t="n"/>
+      <c r="F6" s="30" t="n"/>
+      <c r="G6" s="30" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="n">
+      <c r="A7" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="32" t="inlineStr">
         <is>
           <t>Preparar tartas del día (cheesecake, carrot cake...)</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="C7" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D7" s="29" t="inlineStr">
         <is>
           <t>Pastelero/a</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E7" s="29" t="inlineStr">
         <is>
           <t>06:30</t>
         </is>
       </c>
-      <c r="F7" s="15" t="n"/>
-      <c r="G7" s="15" t="n"/>
+      <c r="F7" s="30" t="n"/>
+      <c r="G7" s="30" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="n">
+      <c r="A8" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="28" t="inlineStr">
         <is>
           <t>Glasear/decorar bollería</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="C8" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D8" s="29" t="inlineStr">
         <is>
           <t>Pastelero/a</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="E8" s="29" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="F8" s="11" t="n"/>
-      <c r="G8" s="11" t="n"/>
+      <c r="F8" s="30" t="n"/>
+      <c r="G8" s="30" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="n">
+      <c r="A9" s="31" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="32" t="inlineStr">
         <is>
           <t>Preparar cookies y brownies</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="C9" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D9" s="29" t="inlineStr">
         <is>
           <t>Pastelero/a</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="29" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="F9" s="15" t="n"/>
-      <c r="G9" s="15" t="n"/>
+      <c r="F9" s="30" t="n"/>
+      <c r="G9" s="30" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="n">
+      <c r="A10" s="27" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="28" t="inlineStr">
         <is>
           <t>Preparar puddings/flanes si aplica</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="C10" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D10" s="29" t="inlineStr">
         <is>
           <t>Pastelero/a</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E10" s="29" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="F10" s="11" t="n"/>
-      <c r="G10" s="11" t="n"/>
+      <c r="F10" s="30" t="n"/>
+      <c r="G10" s="30" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  VITRINA</t>
         </is>
       </c>
+      <c r="B11" s="26" t="n"/>
+      <c r="C11" s="26" t="n"/>
+      <c r="D11" s="26" t="n"/>
+      <c r="E11" s="26" t="n"/>
+      <c r="F11" s="26" t="n"/>
+      <c r="G11" s="26" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="n">
+      <c r="A12" s="27" t="n">
         <v>6</v>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="28" t="inlineStr">
         <is>
           <t>Montar vitrina: colocar piezas con pinzas/guantes</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="C12" s="29" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="D12" s="29" t="inlineStr">
         <is>
           <t>Pastelero/a</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="E12" s="29" t="inlineStr">
         <is>
           <t>07:30</t>
         </is>
       </c>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n"/>
+      <c r="F12" s="30" t="n"/>
+      <c r="G12" s="30" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="n">
+      <c r="A13" s="31" t="n">
         <v>7</v>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="32" t="inlineStr">
         <is>
           <t>Etiquetar cada producto: nombre, precio, alérgenos</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C13" s="29" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="D13" s="29" t="inlineStr">
         <is>
           <t>Pastelero/a</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
+      <c r="E13" s="29" t="inlineStr">
         <is>
           <t>07:30</t>
         </is>
       </c>
-      <c r="F13" s="15" t="n"/>
-      <c r="G13" s="15" t="n"/>
+      <c r="F13" s="30" t="n"/>
+      <c r="G13" s="30" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="20" t="n">
+      <c r="A14" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Verificar temperatura de vitrina refrigerada</t>
-        </is>
-      </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="B14" s="28" t="inlineStr">
+        <is>
+          <t>Verificar temperatura de vitrina refrigerada (refrigeración 0-4 °C) — anota la lectura: ____ °C</t>
+        </is>
+      </c>
+      <c r="C14" s="29" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="D14" s="29" t="inlineStr">
         <is>
           <t>Pastelero/a</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="E14" s="29" t="inlineStr">
         <is>
           <t>07:30</t>
         </is>
       </c>
-      <c r="F14" s="11" t="n"/>
-      <c r="G14" s="11" t="n"/>
+      <c r="F14" s="30" t="n"/>
+      <c r="G14" s="30" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="n">
+      <c r="A15" s="31" t="n">
         <v>9</v>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="32" t="inlineStr">
         <is>
           <t>Limpiar cristal de vitrina (interior y exterior)</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="C15" s="29" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="D15" s="29" t="inlineStr">
         <is>
           <t>Pastelero/a</t>
         </is>
       </c>
-      <c r="E15" s="14" t="inlineStr">
+      <c r="E15" s="29" t="inlineStr">
         <is>
           <t>07:30</t>
         </is>
       </c>
-      <c r="F15" s="15" t="n"/>
-      <c r="G15" s="15" t="n"/>
+      <c r="F15" s="30" t="n"/>
+      <c r="G15" s="30" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="n">
+      <c r="A16" s="27" t="n">
         <v>10</v>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="28" t="inlineStr">
         <is>
           <t>Rotar producto: lo de ayer delante, lo nuevo detrás</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C16" s="29" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D16" s="29" t="inlineStr">
         <is>
           <t>Pastelero/a</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="E16" s="29" t="inlineStr">
         <is>
           <t>07:30</t>
         </is>
       </c>
-      <c r="F16" s="11" t="n"/>
-      <c r="G16" s="11" t="n"/>
+      <c r="F16" s="30" t="n"/>
+      <c r="G16" s="30" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  DURANTE EL SERVICIO</t>
         </is>
       </c>
+      <c r="B17" s="26" t="n"/>
+      <c r="C17" s="26" t="n"/>
+      <c r="D17" s="26" t="n"/>
+      <c r="E17" s="26" t="n"/>
+      <c r="F17" s="26" t="n"/>
+      <c r="G17" s="26" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="20" t="n">
+      <c r="A18" s="27" t="n">
         <v>11</v>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="28" t="inlineStr">
         <is>
           <t>Reponer vitrina cuando baje el stock visible</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr">
+      <c r="C18" s="29" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D18" s="10" t="inlineStr">
+      <c r="D18" s="29" t="inlineStr">
         <is>
           <t>Pastelero/a</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="E18" s="29" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F18" s="11" t="n"/>
-      <c r="G18" s="11" t="n"/>
+      <c r="F18" s="30" t="n"/>
+      <c r="G18" s="30" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="21" t="n">
+      <c r="A19" s="31" t="n">
         <v>12</v>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B19" s="32" t="inlineStr">
         <is>
           <t>Retirar producto que no tenga buen aspecto</t>
         </is>
       </c>
-      <c r="C19" s="14" t="inlineStr">
+      <c r="C19" s="29" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D19" s="14" t="inlineStr">
+      <c r="D19" s="29" t="inlineStr">
         <is>
           <t>Pastelero/a</t>
         </is>
       </c>
-      <c r="E19" s="14" t="inlineStr">
+      <c r="E19" s="29" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F19" s="15" t="n"/>
-      <c r="G19" s="15" t="n"/>
+      <c r="F19" s="30" t="n"/>
+      <c r="G19" s="30" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="20" t="n">
+      <c r="A20" s="27" t="n">
         <v>13</v>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="28" t="inlineStr">
         <is>
           <t>Hornear segunda tanda si hay demanda</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
+      <c r="C20" s="29" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D20" s="29" t="inlineStr">
         <is>
           <t>Pastelero/a</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="E20" s="29" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F20" s="11" t="n"/>
-      <c r="G20" s="11" t="n"/>
+      <c r="F20" s="30" t="n"/>
+      <c r="G20" s="30" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="21" t="n">
+      <c r="A21" s="31" t="n">
         <v>14</v>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="32" t="inlineStr">
         <is>
           <t>Controlar stock de platos/bases para emplatar</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr">
+      <c r="C21" s="29" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="D21" s="29" t="inlineStr">
         <is>
           <t>Pastelero/a</t>
         </is>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E21" s="29" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F21" s="15" t="n"/>
-      <c r="G21" s="15" t="n"/>
+      <c r="F21" s="30" t="n"/>
+      <c r="G21" s="30" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  CIERRE VITRINA</t>
         </is>
       </c>
+      <c r="B22" s="26" t="n"/>
+      <c r="C22" s="26" t="n"/>
+      <c r="D22" s="26" t="n"/>
+      <c r="E22" s="26" t="n"/>
+      <c r="F22" s="26" t="n"/>
+      <c r="G22" s="26" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="n">
+      <c r="A23" s="31" t="n">
         <v>15</v>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="32" t="inlineStr">
         <is>
           <t>Retirar todo de la vitrina y guardar en cámara</t>
         </is>
       </c>
-      <c r="C23" s="14" t="inlineStr">
+      <c r="C23" s="29" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="D23" s="29" t="inlineStr">
         <is>
           <t>Pastelero/a</t>
         </is>
       </c>
-      <c r="E23" s="14" t="inlineStr">
+      <c r="E23" s="29" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F23" s="15" t="n"/>
-      <c r="G23" s="15" t="n"/>
+      <c r="F23" s="30" t="n"/>
+      <c r="G23" s="30" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="20" t="n">
+      <c r="A24" s="27" t="n">
         <v>16</v>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="28" t="inlineStr">
         <is>
           <t>Etiquetar sobrantes con fecha</t>
         </is>
       </c>
-      <c r="C24" s="10" t="inlineStr">
+      <c r="C24" s="29" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D24" s="10" t="inlineStr">
+      <c r="D24" s="29" t="inlineStr">
         <is>
           <t>Pastelero/a</t>
         </is>
       </c>
-      <c r="E24" s="10" t="inlineStr">
+      <c r="E24" s="29" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F24" s="11" t="n"/>
-      <c r="G24" s="11" t="n"/>
+      <c r="F24" s="30" t="n"/>
+      <c r="G24" s="30" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="21" t="n">
+      <c r="A25" s="31" t="n">
         <v>17</v>
       </c>
-      <c r="B25" s="13" t="inlineStr">
+      <c r="B25" s="32" t="inlineStr">
         <is>
           <t>Limpiar interior de vitrina</t>
         </is>
       </c>
-      <c r="C25" s="14" t="inlineStr">
+      <c r="C25" s="29" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr">
+      <c r="D25" s="29" t="inlineStr">
         <is>
           <t>Pastelero/a</t>
         </is>
       </c>
-      <c r="E25" s="14" t="inlineStr">
+      <c r="E25" s="29" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F25" s="15" t="n"/>
-      <c r="G25" s="15" t="n"/>
+      <c r="F25" s="30" t="n"/>
+      <c r="G25" s="30" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="20" t="n">
+      <c r="A26" s="27" t="n">
         <v>18</v>
       </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>Anotar lo que se ha vendido vs producido (para ajustar)</t>
-        </is>
-      </c>
-      <c r="C26" s="10" t="inlineStr">
+      <c r="B26" s="28" t="inlineStr">
+        <is>
+          <t>Anotar producción, ventas y MERMA del día (piezas retiradas, regaladas o al personal): es el dato que ajusta la producción de mañana</t>
+        </is>
+      </c>
+      <c r="C26" s="29" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D26" s="10" t="inlineStr">
+      <c r="D26" s="29" t="inlineStr">
         <is>
           <t>Pastelero/a</t>
         </is>
       </c>
-      <c r="E26" s="10" t="inlineStr">
+      <c r="E26" s="29" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F26" s="11" t="n"/>
-      <c r="G26" s="11" t="n"/>
+      <c r="F26" s="30" t="n"/>
+      <c r="G26" s="30" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="21" t="n">
+      <c r="A27" s="31" t="n">
         <v>19</v>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="32" t="inlineStr">
         <is>
           <t>Preparar lista de producción para mañana</t>
         </is>
       </c>
-      <c r="C27" s="14" t="inlineStr">
+      <c r="C27" s="29" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D27" s="14" t="inlineStr">
+      <c r="D27" s="29" t="inlineStr">
         <is>
           <t>Pastelero/a</t>
         </is>
       </c>
-      <c r="E27" s="14" t="inlineStr">
+      <c r="E27" s="29" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F27" s="15" t="n"/>
-      <c r="G27" s="15" t="n"/>
-    </row>
-    <row r="28"/>
+      <c r="F27" s="30" t="n"/>
+      <c r="G27" s="30" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="33" t="n"/>
+      <c r="B28" s="34" t="n"/>
+      <c r="C28" s="29" t="n"/>
+      <c r="D28" s="29" t="n"/>
+      <c r="E28" s="29" t="n"/>
+      <c r="F28" s="30" t="n"/>
+      <c r="G28" s="30" t="n"/>
+    </row>
     <row r="29">
-      <c r="C29" s="16" t="inlineStr">
-        <is>
-          <t>Completadas:</t>
-        </is>
-      </c>
-      <c r="D29" s="17">
-        <f>COUNTIF(F5:F27,"✓")</f>
+      <c r="A29" s="33" t="n"/>
+      <c r="B29" s="34" t="n"/>
+      <c r="C29" s="29" t="n"/>
+      <c r="D29" s="29" t="n"/>
+      <c r="E29" s="29" t="n"/>
+      <c r="F29" s="30" t="n"/>
+      <c r="G29" s="30" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="33" t="n"/>
+      <c r="B30" s="34" t="n"/>
+      <c r="C30" s="29" t="n"/>
+      <c r="D30" s="29" t="n"/>
+      <c r="E30" s="29" t="n"/>
+      <c r="F30" s="30" t="n"/>
+      <c r="G30" s="30" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="33" t="n"/>
+      <c r="B31" s="34" t="n"/>
+      <c r="C31" s="29" t="n"/>
+      <c r="D31" s="29" t="n"/>
+      <c r="E31" s="29" t="n"/>
+      <c r="F31" s="30" t="n"/>
+      <c r="G31" s="30" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="33" t="n"/>
+      <c r="B32" s="34" t="n"/>
+      <c r="C32" s="29" t="n"/>
+      <c r="D32" s="29" t="n"/>
+      <c r="E32" s="29" t="n"/>
+      <c r="F32" s="30" t="n"/>
+      <c r="G32" s="30" t="n"/>
+    </row>
+    <row r="33"/>
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>Tareas completadas:</t>
+        </is>
+      </c>
+      <c r="D34" s="17">
+        <f>COUNTIFS(B5:B32,"?*",F5:F32,"✓")</f>
         <v>0.0</v>
       </c>
-      <c r="E29" s="16" t="inlineStr">
+      <c r="E34" s="16" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="F29">
-        <f>COUNTIF(B5:B27,"?*")</f>
+      <c r="F34">
+        <f>COUNTIF(B5:B32,"?*")-COUNTIF(F5:F32,"N/A")</f>
         <v>19.0</v>
       </c>
     </row>
-    <row r="30"/>
-    <row r="31">
-      <c r="A31" s="18" t="inlineStr">
+    <row r="35"/>
+    <row r="36">
+      <c r="A36" s="18" t="inlineStr">
         <is>
           <t>Firma encargado/a: _________________________    Hora: _________</t>
         </is>
       </c>
     </row>
-    <row r="32"/>
-    <row r="33">
-      <c r="A33" s="19" t="inlineStr">
-        <is>
-          <t>— Kit de Tareas Recurrentes: Cafetería / Brunch · AI Chef Pro · aichef.pro —</t>
+    <row r="37"/>
+    <row r="38">
+      <c r="A38" s="19" t="inlineStr">
+        <is>
+          <t>— Kit de Tareas Recurrentes · Cafetería / Brunch · AI Chef Pro · aichef.pro</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="0"/>
+  <mergeCells count="9">
+    <mergeCell ref="A36:G36"/>
+    <mergeCell ref="A17:G17"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A33:G33"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="A17:G17"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A34:C34"/>
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="A11:G11"/>
-    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A38:G38"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:G27">
+  <conditionalFormatting sqref="A5:G32">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$F5="✓"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F6 F7 F8 F9 F10 F12 F13 F14 F15 F16 F18 F19 F20 F21 F23 F24 F25 F26 F27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F6 F7 F8 F9 F10 F12 F13 F14 F15 F16 F18 F19 F20 F21 F23 F24 F25 F26 F27 F28 F29 F30 F31 F32" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." type="list" errorStyle="stop">
       <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>